<commit_message>
final fixes for scaffold parser
</commit_message>
<xml_diff>
--- a/tests/ProcessCore.Tests/TestObjects/fct_stri_study.xlsx
+++ b/tests/ProcessCore.Tests/TestObjects/fct_stri_study.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A688A044-57B4-49A1-BBEA-16846CFD1208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="18030" yWindow="3490" windowWidth="29580" windowHeight="16780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="isa_study" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="plant_material" state="visible" r:id="rId5"/>
+    <sheet name="isa_study" sheetId="1" r:id="rId1"/>
+    <sheet name="plant_material" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="197">
   <si>
     <t>STUDY</t>
   </si>
@@ -513,9 +517,6 @@
   </si>
   <si>
     <t>28 days after germination</t>
-  </si>
-  <si>
-    <t>user-specific</t>
   </si>
   <si>
     <t/>
@@ -611,14 +612,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -661,8 +662,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="annotationTable0" displayName="annotationTable0" ref="A1:AT7" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:AT7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="annotationTable0" displayName="annotationTable0" ref="A1:AT7">
+  <autoFilter ref="A1:AT7" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -711,52 +712,52 @@
     <filterColumn colId="45" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="46">
-    <tableColumn id="1" name="Input [Source Name]" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Protocol Type" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Term Source REF (DPBO:1000161)" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Term Accession Number (DPBO:1000161)" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Protocol REF" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Characteristic [organism]" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Term Source REF (OBI:0100026)" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Term Accession Number (OBI:0100026)" totalsRowFunction="none"/>
-    <tableColumn id="9" name="Characteristic [organism part]" totalsRowFunction="none"/>
-    <tableColumn id="10" name="Term Source REF (EFO:0000635)" totalsRowFunction="none"/>
-    <tableColumn id="11" name="Term Accession Number (EFO:0000635)" totalsRowFunction="none"/>
-    <tableColumn id="12" name="Characteristic [plant age]" totalsRowFunction="none"/>
-    <tableColumn id="13" name="Term Source REF (DPBO:0000033)" totalsRowFunction="none"/>
-    <tableColumn id="14" name="Term Accession Number (DPBO:0000033)" totalsRowFunction="none"/>
-    <tableColumn id="15" name="Parameter [growth day length]" totalsRowFunction="none"/>
-    <tableColumn id="16" name="Term Source REF (DPBO:0000041)" totalsRowFunction="none"/>
-    <tableColumn id="17" name="Term Accession Number (DPBO:0000041)" totalsRowFunction="none"/>
-    <tableColumn id="18" name="Parameter [light intensity exposure]" totalsRowFunction="none"/>
-    <tableColumn id="19" name="Unit" totalsRowFunction="none"/>
-    <tableColumn id="20" name="Term Source REF (PECO:0007224)" totalsRowFunction="none"/>
-    <tableColumn id="21" name="Term Accession Number (PECO:0007224)" totalsRowFunction="none"/>
-    <tableColumn id="22" name="Parameter [humidity day]" totalsRowFunction="none"/>
-    <tableColumn id="23" name="Unit " totalsRowFunction="none"/>
-    <tableColumn id="24" name="Term Source REF (DPBO:0000005)" totalsRowFunction="none"/>
-    <tableColumn id="25" name="Term Accession Number (DPBO:0000005)" totalsRowFunction="none"/>
-    <tableColumn id="26" name="Parameter [temperature day]" totalsRowFunction="none"/>
-    <tableColumn id="27" name="Unit  " totalsRowFunction="none"/>
-    <tableColumn id="28" name="Term Source REF (DPBO:0000007)" totalsRowFunction="none"/>
-    <tableColumn id="29" name="Term Accession Number (DPBO:0000007)" totalsRowFunction="none"/>
-    <tableColumn id="30" name="Parameter [temperature night]" totalsRowFunction="none"/>
-    <tableColumn id="31" name="Unit   " totalsRowFunction="none"/>
-    <tableColumn id="32" name="Term Source REF (DPBO:0000008)" totalsRowFunction="none"/>
-    <tableColumn id="33" name="Term Accession Number (DPBO:0000008)" totalsRowFunction="none"/>
-    <tableColumn id="34" name="Factor [watering exposure]" totalsRowFunction="none"/>
-    <tableColumn id="35" name="Term Source REF (PECO:0007383)" totalsRowFunction="none"/>
-    <tableColumn id="36" name="Term Accession Number (PECO:0007383)" totalsRowFunction="none"/>
-    <tableColumn id="37" name="Factor [Timepoint]" totalsRowFunction="none"/>
-    <tableColumn id="38" name="Term Source REF (NCIT:C68568)" totalsRowFunction="none"/>
-    <tableColumn id="39" name="Term Accession Number (NCIT:C68568)" totalsRowFunction="none"/>
-    <tableColumn id="40" name="Factor [timepoint-ZT]" totalsRowFunction="none"/>
-    <tableColumn id="41" name="Term Source REF ()" totalsRowFunction="none"/>
-    <tableColumn id="42" name="Term Accession Number ()" totalsRowFunction="none"/>
-    <tableColumn id="43" name="Factor [Photosynthesis mode]" totalsRowFunction="none"/>
-    <tableColumn id="44" name="Term Source REF () " totalsRowFunction="none"/>
-    <tableColumn id="45" name="Term Accession Number () " totalsRowFunction="none"/>
-    <tableColumn id="46" name="Output [Sample Name]" totalsRowFunction="none"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Input [Source Name]" totalsRowLabel="Total"/>
+    <tableColumn id="47" xr3:uid="{CDA4FC61-214C-4B45-AA8A-1545992A8E88}" name="Protocol REF"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Protocol Type"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Term Source REF (DPBO:1000161)"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Term Accession Number (DPBO:1000161)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Characteristic [organism]"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Term Source REF (OBI:0100026)"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Term Accession Number (OBI:0100026)"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Characteristic [organism part]"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Term Source REF (EFO:0000635)"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Term Accession Number (EFO:0000635)"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Characteristic [plant age]"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Term Source REF (DPBO:0000033)"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Term Accession Number (DPBO:0000033)"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Parameter [growth day length]"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Term Source REF (DPBO:0000041)"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Term Accession Number (DPBO:0000041)"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Parameter [light intensity exposure]"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Unit"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Term Source REF (PECO:0007224)"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Term Accession Number (PECO:0007224)"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Parameter [humidity day]"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Unit "/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Term Source REF (DPBO:0000005)"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Term Accession Number (DPBO:0000005)"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Parameter [temperature day]"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Unit  "/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Term Source REF (DPBO:0000007)"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Term Accession Number (DPBO:0000007)"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Parameter [temperature night]"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Unit   "/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Term Source REF (DPBO:0000008)"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Term Accession Number (DPBO:0000008)"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Factor [watering exposure]"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Term Source REF (PECO:0007383)"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Term Accession Number (PECO:0007383)"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Factor [Timepoint]"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Term Source REF (NCIT:C68568)"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Term Accession Number (NCIT:C68568)"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Factor [timepoint-ZT]"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Term Source REF ()"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Term Accession Number ()"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Factor [Photosynthesis mode]"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Term Source REF () "/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Term Accession Number () "/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Output [Sample Name]"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1058,16 +1059,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E64"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1075,7 +1076,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1083,7 +1084,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1091,17 +1092,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1109,12 +1110,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1130,7 +1131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1138,52 +1139,52 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1200,7 +1201,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1217,7 +1218,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1228,7 +1229,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -1239,12 +1240,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -1258,17 +1259,17 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>49</v>
       </c>
@@ -1279,7 +1280,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -1287,7 +1288,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>54</v>
       </c>
@@ -1295,7 +1296,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>55</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>57</v>
       </c>
@@ -1311,7 +1312,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>59</v>
       </c>
@@ -1319,7 +1320,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>60</v>
       </c>
@@ -1327,7 +1328,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>62</v>
       </c>
@@ -1341,12 +1342,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>67</v>
       </c>
@@ -1354,7 +1355,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -1362,7 +1363,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>71</v>
       </c>
@@ -1370,7 +1371,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -1378,22 +1379,22 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>78</v>
       </c>
@@ -1401,7 +1402,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>80</v>
       </c>
@@ -1409,7 +1410,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>82</v>
       </c>
@@ -1417,32 +1418,32 @@
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>89</v>
       </c>
@@ -1453,7 +1454,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>92</v>
       </c>
@@ -1464,12 +1465,12 @@
         <v>94</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>96</v>
       </c>
@@ -1477,7 +1478,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>98</v>
       </c>
@@ -1485,12 +1486,12 @@
         <v>99</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>101</v>
       </c>
@@ -1501,7 +1502,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>104</v>
       </c>
@@ -1512,7 +1513,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>107</v>
       </c>
@@ -1523,7 +1524,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>110</v>
       </c>
@@ -1534,7 +1535,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>113</v>
       </c>
@@ -1545,7 +1546,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>115</v>
       </c>
@@ -1555,30 +1556,30 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AT7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>117</v>
       </c>
       <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
         <v>118</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>119</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>120</v>
-      </c>
-      <c r="E1" t="s">
-        <v>121</v>
       </c>
       <c r="F1" t="s">
         <v>122</v>
@@ -1704,21 +1705,21 @@
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>159</v>
       </c>
       <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
         <v>70</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>74</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>72</v>
-      </c>
-      <c r="E2" t="s">
-        <v>68</v>
       </c>
       <c r="F2" t="s">
         <v>160</v>
@@ -1741,124 +1742,106 @@
       <c r="L2" t="s">
         <v>166</v>
       </c>
-      <c r="M2" t="s">
-        <v>167</v>
-      </c>
       <c r="N2" t="s">
+        <v>167</v>
+      </c>
+      <c r="O2" t="s">
         <v>168</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
+        <v>167</v>
+      </c>
+      <c r="R2" t="s">
         <v>169</v>
       </c>
-      <c r="P2" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>168</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>170</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>171</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>172</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>173</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>174</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y2" t="s">
         <v>175</v>
       </c>
-      <c r="X2" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>176</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>177</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC2" t="s">
         <v>178</v>
       </c>
-      <c r="AB2" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>179</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AH2" t="s">
         <v>180</v>
       </c>
-      <c r="AE2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH2" t="s">
+      <c r="AJ2" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK2" t="s">
         <v>181</v>
       </c>
-      <c r="AI2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK2" t="s">
+      <c r="AM2" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN2" t="s">
         <v>182</v>
       </c>
-      <c r="AL2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN2" t="s">
+      <c r="AP2" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ2" t="s">
         <v>183</v>
       </c>
-      <c r="AO2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ2" t="s">
+      <c r="AS2" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT2" t="s">
         <v>184</v>
       </c>
-      <c r="AR2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AT2" t="s">
+    </row>
+    <row r="3" spans="1:46" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>186</v>
-      </c>
       <c r="B3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" t="s">
         <v>70</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>74</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>72</v>
-      </c>
-      <c r="E3" t="s">
-        <v>68</v>
       </c>
       <c r="F3" t="s">
         <v>160</v>
@@ -1881,124 +1864,106 @@
       <c r="L3" t="s">
         <v>166</v>
       </c>
-      <c r="M3" t="s">
-        <v>167</v>
-      </c>
       <c r="N3" t="s">
+        <v>167</v>
+      </c>
+      <c r="O3" t="s">
         <v>168</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
+        <v>167</v>
+      </c>
+      <c r="R3" t="s">
         <v>169</v>
       </c>
-      <c r="P3" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>168</v>
-      </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>170</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>171</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>172</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>173</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>174</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y3" t="s">
         <v>175</v>
       </c>
-      <c r="X3" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>176</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>177</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC3" t="s">
         <v>178</v>
       </c>
-      <c r="AB3" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>179</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>178</v>
+      </c>
+      <c r="AH3" t="s">
         <v>180</v>
       </c>
-      <c r="AE3" t="s">
-        <v>178</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH3" t="s">
+      <c r="AJ3" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK3" t="s">
         <v>181</v>
       </c>
-      <c r="AI3" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK3" t="s">
+      <c r="AM3" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN3" t="s">
         <v>182</v>
       </c>
-      <c r="AL3" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN3" t="s">
+      <c r="AP3" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ3" t="s">
         <v>183</v>
       </c>
-      <c r="AO3" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>184</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>167</v>
-      </c>
       <c r="AS3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AT3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:46" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>188</v>
-      </c>
       <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
         <v>70</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>74</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>72</v>
-      </c>
-      <c r="E4" t="s">
-        <v>68</v>
       </c>
       <c r="F4" t="s">
         <v>160</v>
@@ -2021,124 +1986,106 @@
       <c r="L4" t="s">
         <v>166</v>
       </c>
-      <c r="M4" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" t="s">
+        <v>167</v>
+      </c>
+      <c r="O4" t="s">
         <v>168</v>
       </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
+        <v>167</v>
+      </c>
+      <c r="R4" t="s">
         <v>169</v>
       </c>
-      <c r="P4" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>168</v>
-      </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>170</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>171</v>
       </c>
-      <c r="T4" t="s">
+      <c r="U4" t="s">
         <v>172</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>173</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>174</v>
       </c>
-      <c r="W4" t="s">
+      <c r="X4" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y4" t="s">
         <v>175</v>
       </c>
-      <c r="X4" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>176</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>177</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AB4" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC4" t="s">
         <v>178</v>
       </c>
-      <c r="AB4" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>179</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>178</v>
+      </c>
+      <c r="AH4" t="s">
         <v>180</v>
       </c>
-      <c r="AE4" t="s">
-        <v>178</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH4" t="s">
+      <c r="AJ4" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK4" t="s">
         <v>181</v>
       </c>
-      <c r="AI4" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK4" t="s">
+      <c r="AM4" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN4" t="s">
         <v>182</v>
       </c>
-      <c r="AL4" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN4" t="s">
+      <c r="AP4" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ4" t="s">
         <v>183</v>
       </c>
-      <c r="AO4" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP4" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>184</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>167</v>
-      </c>
       <c r="AS4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AT4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:46" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>190</v>
-      </c>
       <c r="B5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" t="s">
         <v>70</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>74</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>72</v>
-      </c>
-      <c r="E5" t="s">
-        <v>68</v>
       </c>
       <c r="F5" t="s">
         <v>160</v>
@@ -2161,124 +2108,106 @@
       <c r="L5" t="s">
         <v>166</v>
       </c>
-      <c r="M5" t="s">
-        <v>167</v>
-      </c>
       <c r="N5" t="s">
+        <v>167</v>
+      </c>
+      <c r="O5" t="s">
         <v>168</v>
       </c>
-      <c r="O5" t="s">
+      <c r="Q5" t="s">
+        <v>167</v>
+      </c>
+      <c r="R5" t="s">
         <v>169</v>
       </c>
-      <c r="P5" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>168</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>170</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>171</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>172</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>173</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>174</v>
       </c>
-      <c r="W5" t="s">
+      <c r="X5" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y5" t="s">
         <v>175</v>
       </c>
-      <c r="X5" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>176</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>177</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AB5" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC5" t="s">
         <v>178</v>
       </c>
-      <c r="AB5" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>179</v>
       </c>
-      <c r="AD5" t="s">
-        <v>180</v>
-      </c>
       <c r="AE5" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG5" t="s">
         <v>178</v>
       </c>
-      <c r="AF5" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>179</v>
-      </c>
       <c r="AH5" t="s">
+        <v>190</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>182</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ5" t="s">
         <v>191</v>
       </c>
-      <c r="AI5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>182</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>183</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ5" t="s">
+      <c r="AS5" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT5" t="s">
         <v>192</v>
       </c>
-      <c r="AR5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AS5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AT5" t="s">
+    </row>
+    <row r="6" spans="1:46" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>194</v>
-      </c>
       <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
         <v>70</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>74</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>72</v>
-      </c>
-      <c r="E6" t="s">
-        <v>68</v>
       </c>
       <c r="F6" t="s">
         <v>160</v>
@@ -2301,124 +2230,106 @@
       <c r="L6" t="s">
         <v>166</v>
       </c>
-      <c r="M6" t="s">
-        <v>167</v>
-      </c>
       <c r="N6" t="s">
+        <v>167</v>
+      </c>
+      <c r="O6" t="s">
         <v>168</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q6" t="s">
+        <v>167</v>
+      </c>
+      <c r="R6" t="s">
         <v>169</v>
       </c>
-      <c r="P6" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>168</v>
-      </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>170</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>171</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>172</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>173</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>174</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y6" t="s">
         <v>175</v>
       </c>
-      <c r="X6" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>176</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>177</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC6" t="s">
         <v>178</v>
       </c>
-      <c r="AB6" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>179</v>
       </c>
-      <c r="AD6" t="s">
-        <v>180</v>
-      </c>
       <c r="AE6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG6" t="s">
         <v>178</v>
       </c>
-      <c r="AF6" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>179</v>
-      </c>
       <c r="AH6" t="s">
+        <v>190</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>181</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>182</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ6" t="s">
         <v>191</v>
       </c>
-      <c r="AI6" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>182</v>
-      </c>
-      <c r="AL6" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM6" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN6" t="s">
-        <v>183</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP6" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ6" t="s">
-        <v>192</v>
-      </c>
-      <c r="AR6" t="s">
-        <v>167</v>
-      </c>
       <c r="AS6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AT6" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:46" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>196</v>
-      </c>
       <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" t="s">
         <v>70</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>74</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>72</v>
-      </c>
-      <c r="E7" t="s">
-        <v>68</v>
       </c>
       <c r="F7" t="s">
         <v>160</v>
@@ -2441,112 +2352,94 @@
       <c r="L7" t="s">
         <v>166</v>
       </c>
-      <c r="M7" t="s">
-        <v>167</v>
-      </c>
       <c r="N7" t="s">
+        <v>167</v>
+      </c>
+      <c r="O7" t="s">
         <v>168</v>
       </c>
-      <c r="O7" t="s">
+      <c r="Q7" t="s">
+        <v>167</v>
+      </c>
+      <c r="R7" t="s">
         <v>169</v>
       </c>
-      <c r="P7" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>168</v>
-      </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>170</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>171</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>172</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>173</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>174</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y7" t="s">
         <v>175</v>
       </c>
-      <c r="X7" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>176</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>177</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC7" t="s">
         <v>178</v>
       </c>
-      <c r="AB7" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>179</v>
       </c>
-      <c r="AD7" t="s">
-        <v>180</v>
-      </c>
       <c r="AE7" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG7" t="s">
         <v>178</v>
       </c>
-      <c r="AF7" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>179</v>
-      </c>
       <c r="AH7" t="s">
+        <v>190</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>181</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>182</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AQ7" t="s">
         <v>191</v>
       </c>
-      <c r="AI7" t="s">
-        <v>167</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>168</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>182</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>167</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>168</v>
-      </c>
-      <c r="AN7" t="s">
-        <v>183</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>167</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ7" t="s">
-        <v>192</v>
-      </c>
-      <c r="AR7" t="s">
-        <v>167</v>
-      </c>
       <c r="AS7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AT7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>